<commit_message>
updated the presenters order
</commit_message>
<xml_diff>
--- a/website_data.xlsx
+++ b/website_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://crwindia-my.sharepoint.com/personal/fin_crwi_org_in/Documents/Jomit_clean/crwisymposium/crwisymposium-new7-4-26/crwisymposium-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{43A54E2A-C15B-4049-9416-409D91501929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D88676A8-7DEE-4B9E-A475-47AE74C7ACAE}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="13_ncr:1_{43A54E2A-C15B-4049-9416-409D91501929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E678AA4-A905-489F-82E3-5207D6D419EA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="747" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="747" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global_Settings" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
     <author>Religiouswomen India</author>
   </authors>
   <commentList>
-    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{BF718063-9DB4-4990-8D93-69F27DF27465}">
+    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{BF718063-9DB4-4990-8D93-69F27DF27465}">
       <text>
         <r>
           <rPr>
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="548">
   <si>
     <t>Setting_Key</t>
   </si>
@@ -740,9 +740,6 @@
     <t>Addressing psychological well-being, intercultural living, and the responsible use of technology</t>
   </si>
   <si>
-    <t>Intercultural and intergenerational community living</t>
-  </si>
-  <si>
     <t>Reimagining structures to integrate spiritual, human, intellectual, and pastoral dimensions.</t>
   </si>
   <si>
@@ -1067,9 +1064,6 @@
     <t>images/Trustees/3.jpg</t>
   </si>
   <si>
-    <t>images/Trustees/4.jpg</t>
-  </si>
-  <si>
     <t>images/Trustees/5.jpg</t>
   </si>
   <si>
@@ -1541,9 +1535,6 @@
     <t>Fr. Dr. Johnson</t>
   </si>
   <si>
-    <t>Fr. V. Antony Bhyju</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sr. Dr. Mary Paul </t>
   </si>
   <si>
@@ -1739,9 +1730,6 @@
     <t>images/Speakers/Bibina.jpg</t>
   </si>
   <si>
-    <t>Dr. Fr. Dominic</t>
-  </si>
-  <si>
     <t>Dr. Fr. Joye James</t>
   </si>
   <si>
@@ -1749,6 +1737,22 @@
   </si>
   <si>
     <t>Member of the Congregation of the Apostolic Carmel, Sr. Lavina Rodrigues AC is a trained formator with experience accompanying Aspirants, Novices, and Juniors, and holds an MA in English with extensive teaching and formative leadership experience.</t>
+  </si>
+  <si>
+    <t>Unity in Diversity: A Convergent Walking in a Divergent Context
+A Critical Analysis of Synodal, Inter-Congregational, and Inter-Cultural Formation in Theological Education at Institute Mater Dei (IMD), Goa, India</t>
+  </si>
+  <si>
+    <t>Fr. Augustin  Bhayju</t>
+  </si>
+  <si>
+    <t>Fr. Mathew Abraham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr. Ronald </t>
+  </si>
+  <si>
+    <t>Logos/Logo 6.jpg</t>
   </si>
 </sst>
 </file>
@@ -1901,6 +1905,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2370,7 +2378,7 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -2381,7 +2389,7 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -2403,13 +2411,13 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>0</v>
@@ -2418,7 +2426,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="N9" t="s">
         <v>19</v>
@@ -2426,36 +2434,36 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B10" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C10" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E10" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="H10" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="I10" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="E11" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="H11" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="I11" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
@@ -2463,19 +2471,19 @@
         <v>0</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E12" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="H12" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="I12" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
@@ -2483,186 +2491,186 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C13" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B14" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B15" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C15" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B16" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C16" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B17" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C17" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B18" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C18" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B19" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C19" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B20" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C20" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B21" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C21" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B22" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C22" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B23" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C23" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B24" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C24" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B25" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C25" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B26" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C26" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B27" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C27" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B28" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="C28" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B29" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="C29" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -2706,13 +2714,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2720,13 +2728,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E3" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -2734,13 +2742,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -2748,13 +2756,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C5" t="s">
+        <v>434</v>
+      </c>
+      <c r="E5" t="s">
         <v>435</v>
-      </c>
-      <c r="C5" t="s">
-        <v>436</v>
-      </c>
-      <c r="E5" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.4">
@@ -2762,13 +2770,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C6" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="E6" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.4">
@@ -2776,13 +2784,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C7" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="E7" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -2790,13 +2798,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C8" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="E8" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2804,13 +2812,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C9" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E9" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -2858,67 +2866,70 @@
         <v>132</v>
       </c>
       <c r="H1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>28</v>
+      <c r="A2" s="3">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C2" t="s">
-        <v>205</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>207</v>
+        <v>463</v>
       </c>
       <c r="E2" t="s">
         <v>88</v>
       </c>
       <c r="F2" t="s">
-        <v>304</v>
+        <v>479</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>263</v>
+        <v>535</v>
       </c>
       <c r="H2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>40</v>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>466</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
+      </c>
+      <c r="D3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E3" t="s">
+        <v>88</v>
       </c>
       <c r="F3" t="s">
-        <v>276</v>
+        <v>303</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>133</v>
+        <v>262</v>
       </c>
       <c r="H3" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="62" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>43</v>
+      <c r="A4" s="3">
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D4" t="s">
         <v>209</v>
@@ -2927,24 +2938,24 @@
         <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="H4" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="62" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>46</v>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="C5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D5" t="s">
         <v>210</v>
@@ -2953,143 +2964,143 @@
         <v>88</v>
       </c>
       <c r="F5" t="s">
-        <v>277</v>
+        <v>307</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>546</v>
+        <v>522</v>
       </c>
       <c r="H5" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>476</v>
+      <c r="B6" t="s">
+        <v>202</v>
       </c>
       <c r="C6" t="s">
-        <v>334</v>
+        <v>457</v>
       </c>
       <c r="D6" t="s">
-        <v>335</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>91</v>
+        <v>211</v>
+      </c>
+      <c r="E6" t="s">
+        <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>545</v>
+        <v>277</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>133</v>
+        <v>263</v>
       </c>
       <c r="H6" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="C7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>211</v>
+        <v>543</v>
       </c>
       <c r="E7" t="s">
         <v>88</v>
       </c>
       <c r="F7" t="s">
-        <v>308</v>
+        <v>276</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>525</v>
+        <v>542</v>
       </c>
       <c r="H7" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>202</v>
+        <v>416</v>
       </c>
       <c r="C8" t="s">
-        <v>459</v>
+        <v>422</v>
       </c>
       <c r="D8" t="s">
-        <v>212</v>
+        <v>453</v>
       </c>
       <c r="E8" t="s">
         <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>278</v>
+        <v>454</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>264</v>
+        <v>530</v>
       </c>
       <c r="H8" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>478</v>
+      <c r="B9" s="11" t="s">
+        <v>545</v>
       </c>
       <c r="C9" t="s">
-        <v>225</v>
+        <v>133</v>
       </c>
       <c r="D9" t="s">
-        <v>221</v>
+        <v>463</v>
       </c>
       <c r="E9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F9" t="s">
-        <v>279</v>
+        <v>425</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>265</v>
+        <v>133</v>
       </c>
       <c r="H9" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="C10" t="s">
-        <v>206</v>
+        <v>455</v>
       </c>
       <c r="D10" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="E10" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F10" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="H10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3097,103 +3108,103 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="C11" t="s">
-        <v>459</v>
+        <v>215</v>
       </c>
       <c r="D11" t="s">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="E11" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F11" t="s">
-        <v>281</v>
+        <v>428</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="H11" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>325</v>
+      <c r="B12" t="s">
+        <v>327</v>
       </c>
       <c r="C12" t="s">
-        <v>133</v>
+        <v>224</v>
       </c>
       <c r="D12" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="E12" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F12" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>133</v>
+        <v>527</v>
       </c>
       <c r="H12" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
       <c r="C13" t="s">
-        <v>226</v>
+        <v>458</v>
       </c>
       <c r="D13" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="E13" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>526</v>
+        <v>270</v>
       </c>
       <c r="H13" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
-        <v>540</v>
+      <c r="B14" s="11" t="s">
+        <v>546</v>
       </c>
       <c r="C14" t="s">
-        <v>227</v>
+        <v>133</v>
       </c>
       <c r="D14" t="s">
-        <v>222</v>
+        <v>463</v>
       </c>
       <c r="E14" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F14" t="s">
-        <v>283</v>
+        <v>425</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>266</v>
+        <v>133</v>
       </c>
       <c r="H14" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
@@ -3201,25 +3212,25 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C15" t="s">
-        <v>203</v>
+        <v>258</v>
       </c>
       <c r="D15" t="s">
-        <v>228</v>
+        <v>260</v>
       </c>
       <c r="E15" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="F15" t="s">
-        <v>415</v>
+        <v>299</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>532</v>
+        <v>274</v>
       </c>
       <c r="H15" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3227,51 +3238,51 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>469</v>
+        <v>324</v>
       </c>
       <c r="C16" t="s">
-        <v>470</v>
+        <v>257</v>
       </c>
       <c r="D16" t="s">
-        <v>229</v>
+        <v>326</v>
       </c>
       <c r="E16" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="F16" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="H16" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="93" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>461</v>
+        <v>255</v>
       </c>
       <c r="C17" t="s">
-        <v>475</v>
+        <v>226</v>
       </c>
       <c r="D17" t="s">
-        <v>323</v>
+        <v>254</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="F17" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>471</v>
+        <v>524</v>
       </c>
       <c r="H17" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3279,25 +3290,25 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>223</v>
+        <v>256</v>
       </c>
       <c r="C18" t="s">
-        <v>458</v>
+        <v>259</v>
       </c>
       <c r="D18" t="s">
-        <v>230</v>
+        <v>325</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="F18" t="s">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>268</v>
+        <v>306</v>
       </c>
       <c r="H18" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3305,25 +3316,25 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>224</v>
+        <v>465</v>
       </c>
       <c r="C19" t="s">
-        <v>459</v>
+        <v>133</v>
       </c>
       <c r="D19" t="s">
-        <v>231</v>
+        <v>463</v>
       </c>
       <c r="E19" t="s">
         <v>91</v>
       </c>
       <c r="F19" t="s">
-        <v>287</v>
+        <v>480</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>269</v>
+        <v>531</v>
       </c>
       <c r="H19" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
@@ -3331,100 +3342,103 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>232</v>
+        <v>472</v>
       </c>
       <c r="C20" t="s">
-        <v>457</v>
+        <v>203</v>
       </c>
       <c r="D20" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="E20" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>288</v>
+        <v>413</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="H20" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>206</v>
+      <c r="B21" t="s">
+        <v>467</v>
+      </c>
+      <c r="C21" t="s">
+        <v>468</v>
       </c>
       <c r="D21" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F21" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>133</v>
+        <v>266</v>
       </c>
       <c r="H21" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
-        <v>329</v>
+      <c r="B22" s="11" t="s">
+        <v>474</v>
       </c>
       <c r="C22" t="s">
-        <v>225</v>
+        <v>332</v>
       </c>
       <c r="D22" t="s">
-        <v>241</v>
-      </c>
-      <c r="E22" t="s">
-        <v>94</v>
+        <v>333</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>290</v>
+        <v>541</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>530</v>
+        <v>133</v>
       </c>
       <c r="H22" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>238</v>
+      <c r="B23" t="s">
+        <v>223</v>
+      </c>
+      <c r="C23" t="s">
+        <v>457</v>
+      </c>
+      <c r="D23" t="s">
+        <v>230</v>
+      </c>
+      <c r="E23" t="s">
+        <v>91</v>
       </c>
       <c r="F23" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>133</v>
+        <v>268</v>
       </c>
       <c r="H23" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3432,25 +3446,25 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>234</v>
+        <v>459</v>
       </c>
       <c r="C24" t="s">
-        <v>216</v>
+        <v>473</v>
       </c>
       <c r="D24" t="s">
-        <v>239</v>
+        <v>321</v>
       </c>
       <c r="E24" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F24" t="s">
-        <v>430</v>
+        <v>284</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>270</v>
+        <v>469</v>
       </c>
       <c r="H24" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3458,117 +3472,129 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>235</v>
+        <v>222</v>
       </c>
       <c r="C25" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="D25" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="E25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F25" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="H25" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" t="s">
-        <v>242</v>
+      <c r="B26" s="11" t="s">
+        <v>540</v>
       </c>
       <c r="C26" t="s">
-        <v>203</v>
+        <v>477</v>
       </c>
       <c r="D26" t="s">
-        <v>249</v>
+        <v>463</v>
       </c>
       <c r="E26" t="s">
         <v>100</v>
       </c>
       <c r="F26" t="s">
-        <v>293</v>
+        <v>481</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>272</v>
+        <v>532</v>
       </c>
       <c r="H26" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>26</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>462</v>
+      <c r="B27" t="s">
+        <v>241</v>
+      </c>
+      <c r="C27" t="s">
+        <v>203</v>
       </c>
       <c r="D27" t="s">
-        <v>324</v>
+        <v>248</v>
       </c>
       <c r="E27" t="s">
         <v>100</v>
       </c>
       <c r="F27" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>133</v>
+        <v>271</v>
       </c>
       <c r="H27" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>133</v>
+      <c r="B28" t="s">
+        <v>328</v>
+      </c>
+      <c r="C28" t="s">
+        <v>245</v>
+      </c>
+      <c r="D28" t="s">
+        <v>249</v>
+      </c>
+      <c r="E28" t="s">
+        <v>100</v>
       </c>
       <c r="F28" t="s">
-        <v>295</v>
+        <v>506</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>133</v>
+        <v>526</v>
       </c>
       <c r="H28" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>133</v>
+      <c r="B29" t="s">
+        <v>243</v>
+      </c>
+      <c r="C29" t="s">
+        <v>247</v>
+      </c>
+      <c r="D29" t="s">
+        <v>252</v>
+      </c>
+      <c r="E29" t="s">
+        <v>100</v>
       </c>
       <c r="F29" t="s">
-        <v>296</v>
+        <v>427</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>133</v>
+        <v>272</v>
       </c>
       <c r="H29" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3576,25 +3602,25 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>330</v>
+        <v>244</v>
       </c>
       <c r="C30" t="s">
-        <v>246</v>
+        <v>206</v>
       </c>
       <c r="D30" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E30" t="s">
         <v>100</v>
       </c>
       <c r="F30" t="s">
-        <v>509</v>
+        <v>297</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>529</v>
+        <v>273</v>
       </c>
       <c r="H30" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
@@ -3602,178 +3628,181 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D31" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E31" t="s">
         <v>100</v>
       </c>
       <c r="F31" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="H31" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="B32" t="s">
-        <v>244</v>
-      </c>
-      <c r="C32" t="s">
-        <v>248</v>
+      <c r="B32" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>460</v>
       </c>
       <c r="D32" t="s">
-        <v>253</v>
+        <v>322</v>
       </c>
       <c r="E32" t="s">
         <v>100</v>
       </c>
       <c r="F32" t="s">
-        <v>429</v>
+        <v>293</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>273</v>
+        <v>133</v>
       </c>
       <c r="H32" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>245</v>
+        <v>478</v>
       </c>
       <c r="C33" t="s">
-        <v>206</v>
+        <v>133</v>
       </c>
       <c r="D33" t="s">
-        <v>252</v>
+        <v>463</v>
       </c>
       <c r="E33" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F33" t="s">
-        <v>298</v>
+        <v>425</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>274</v>
+        <v>133</v>
       </c>
       <c r="H33" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>326</v>
+        <v>214</v>
       </c>
       <c r="C34" t="s">
-        <v>258</v>
+        <v>225</v>
       </c>
       <c r="D34" t="s">
-        <v>328</v>
+        <v>219</v>
       </c>
       <c r="E34" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="F34" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>262</v>
+        <v>523</v>
       </c>
       <c r="H34" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>479</v>
+        <v>537</v>
       </c>
       <c r="C35" t="s">
-        <v>259</v>
+        <v>226</v>
       </c>
       <c r="D35" t="s">
-        <v>261</v>
+        <v>221</v>
       </c>
       <c r="E35" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="F35" t="s">
-        <v>300</v>
+        <v>282</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="H35" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>325</v>
+      <c r="B36" t="s">
+        <v>213</v>
       </c>
       <c r="C36" t="s">
-        <v>133</v>
+        <v>457</v>
       </c>
       <c r="D36" t="s">
-        <v>254</v>
+        <v>217</v>
+      </c>
+      <c r="E36" t="s">
+        <v>97</v>
       </c>
       <c r="F36" t="s">
-        <v>301</v>
+        <v>280</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>133</v>
+        <v>265</v>
       </c>
       <c r="H36" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="93" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>256</v>
+        <v>475</v>
       </c>
       <c r="C37" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D37" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
       <c r="E37" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="F37" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>527</v>
+        <v>264</v>
       </c>
       <c r="H37" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="62" x14ac:dyDescent="0.35">
@@ -3781,25 +3810,25 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>257</v>
+        <v>212</v>
       </c>
       <c r="C38" t="s">
-        <v>260</v>
+        <v>206</v>
       </c>
       <c r="D38" t="s">
-        <v>327</v>
+        <v>216</v>
       </c>
       <c r="E38" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="F38" t="s">
-        <v>303</v>
+        <v>279</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>307</v>
+        <v>533</v>
       </c>
       <c r="H38" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
@@ -3807,181 +3836,160 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>418</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>424</v>
-      </c>
-      <c r="D39" t="s">
-        <v>455</v>
-      </c>
-      <c r="E39" t="s">
-        <v>88</v>
+        <v>133</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>208</v>
       </c>
       <c r="F39" t="s">
-        <v>456</v>
+        <v>275</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>533</v>
+        <v>133</v>
       </c>
       <c r="H39" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>39</v>
       </c>
-      <c r="B40" t="s">
-        <v>466</v>
+      <c r="B40" s="6" t="s">
+        <v>323</v>
       </c>
       <c r="C40" t="s">
         <v>133</v>
       </c>
       <c r="D40" t="s">
-        <v>465</v>
+        <v>218</v>
       </c>
       <c r="E40" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="F40" t="s">
-        <v>482</v>
+        <v>281</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>538</v>
+        <v>133</v>
       </c>
       <c r="H40" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>40</v>
       </c>
-      <c r="B41" t="s">
-        <v>467</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="B41" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D41" t="s">
+        <v>236</v>
+      </c>
+      <c r="E41" t="s">
+        <v>94</v>
+      </c>
+      <c r="F41" t="s">
+        <v>288</v>
+      </c>
+      <c r="G41" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D41" t="s">
-        <v>465</v>
-      </c>
-      <c r="E41" t="s">
-        <v>91</v>
-      </c>
-      <c r="F41" t="s">
-        <v>483</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>534</v>
-      </c>
       <c r="H41" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="B42" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D42" t="s">
-        <v>465</v>
-      </c>
-      <c r="E42" t="s">
-        <v>104</v>
+      <c r="D42" s="1" t="s">
+        <v>237</v>
       </c>
       <c r="F42" t="s">
-        <v>427</v>
+        <v>290</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>133</v>
       </c>
       <c r="H42" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>42</v>
       </c>
-      <c r="B43" s="11" t="s">
-        <v>544</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B43" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D43" t="s">
-        <v>465</v>
-      </c>
-      <c r="E43" t="s">
-        <v>94</v>
-      </c>
       <c r="F43" t="s">
-        <v>427</v>
+        <v>294</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>133</v>
       </c>
       <c r="H43" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="62" x14ac:dyDescent="0.35">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>43</v>
       </c>
-      <c r="B44" s="11" t="s">
-        <v>544</v>
-      </c>
-      <c r="C44" t="s">
-        <v>480</v>
-      </c>
-      <c r="D44" t="s">
-        <v>465</v>
-      </c>
-      <c r="E44" t="s">
-        <v>100</v>
+      <c r="B44" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>133</v>
       </c>
       <c r="F44" t="s">
-        <v>484</v>
+        <v>295</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>535</v>
+        <v>133</v>
       </c>
       <c r="H44" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>44</v>
       </c>
-      <c r="B45" t="s">
-        <v>481</v>
+      <c r="B45" s="6" t="s">
+        <v>323</v>
       </c>
       <c r="C45" t="s">
         <v>133</v>
       </c>
       <c r="D45" t="s">
-        <v>465</v>
-      </c>
-      <c r="E45" t="s">
-        <v>97</v>
+        <v>253</v>
       </c>
       <c r="F45" t="s">
-        <v>427</v>
+        <v>300</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>133</v>
       </c>
       <c r="H45" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -3989,7 +3997,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="G1 A2:A5 E2 A1:D1 F1" numberStoredAsText="1"/>
+    <ignoredError sqref="E3 A1:D1 F1:G1" numberStoredAsText="1"/>
   </ignoredErrors>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
@@ -4208,13 +4216,13 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C2" t="s">
         <v>309</v>
       </c>
-      <c r="C2" t="s">
-        <v>310</v>
-      </c>
       <c r="D2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -4222,13 +4230,13 @@
         <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C3" t="s">
         <v>150</v>
       </c>
       <c r="D3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -4236,13 +4244,13 @@
         <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>154</v>
       </c>
       <c r="D4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -4250,13 +4258,13 @@
         <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C5" t="s">
         <v>158</v>
       </c>
       <c r="D5" t="s">
-        <v>319</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -4264,13 +4272,13 @@
         <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C6" t="s">
         <v>158</v>
       </c>
       <c r="D6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -4278,13 +4286,13 @@
         <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C7" t="s">
         <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -4319,7 +4327,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -4330,7 +4338,7 @@
         <v>185</v>
       </c>
       <c r="C3" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D3" t="s">
         <v>85</v>
@@ -4341,13 +4349,13 @@
         <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C4" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -4358,10 +4366,10 @@
         <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -4372,10 +4380,10 @@
         <v>181</v>
       </c>
       <c r="C6" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -4383,13 +4391,13 @@
         <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C7" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D7" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -4397,13 +4405,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>518</v>
+      </c>
+      <c r="C8" t="s">
+        <v>420</v>
+      </c>
+      <c r="D8" t="s">
         <v>521</v>
-      </c>
-      <c r="C8" t="s">
-        <v>422</v>
-      </c>
-      <c r="D8" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -4411,13 +4419,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C9" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D9" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -4425,13 +4433,13 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C10" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D10" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -4439,13 +4447,13 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>418</v>
+      </c>
+      <c r="C11" t="s">
         <v>420</v>
       </c>
-      <c r="C11" t="s">
-        <v>422</v>
-      </c>
       <c r="D11" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -4453,13 +4461,13 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C12" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D12" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -4467,18 +4475,18 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C13" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D13" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -4486,13 +4494,13 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C15" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D15" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -4500,13 +4508,13 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C16" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D16" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -4514,13 +4522,13 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C17" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D17" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -4528,13 +4536,13 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="C18" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D18" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -4542,13 +4550,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="C19" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D19" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -4556,13 +4564,13 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="C20" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D20" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -4570,13 +4578,13 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="C21" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D21" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -4584,13 +4592,13 @@
         <v>8</v>
       </c>
       <c r="B22" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C22" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D22" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -4598,13 +4606,13 @@
         <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="C23" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D23" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -4612,13 +4620,13 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="C24" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D24" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -4626,13 +4634,13 @@
         <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="C25" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D25" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -4640,13 +4648,13 @@
         <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="C26" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D26" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -4654,13 +4662,13 @@
         <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="C27" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D27" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -4668,13 +4676,13 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="C28" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D28" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -4857,7 +4865,7 @@
         <v>196</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="E10" t="s">
         <v>128</v>
@@ -4957,8 +4965,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="27.4140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -5042,6 +5053,20 @@
       </c>
       <c r="D6" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="3">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -5544,16 +5569,16 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -5561,16 +5586,16 @@
         <v>40</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E3" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -5578,16 +5603,16 @@
         <v>43</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="C4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E4" t="s">
         <v>432</v>
-      </c>
-      <c r="C4" t="s">
-        <v>433</v>
-      </c>
-      <c r="D4" t="s">
-        <v>431</v>
-      </c>
-      <c r="E4" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -5595,16 +5620,16 @@
         <v>46</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -5615,13 +5640,13 @@
         <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D6" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E6" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -5629,16 +5654,16 @@
         <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C7" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="D7" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E7" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -5646,16 +5671,16 @@
         <v>187</v>
       </c>
       <c r="B8" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C8" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="D8" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -5663,16 +5688,16 @@
         <v>191</v>
       </c>
       <c r="B9" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C9" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D9" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E9" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -5680,16 +5705,16 @@
         <v>194</v>
       </c>
       <c r="B10" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C10" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E10" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated speaker and profile section
</commit_message>
<xml_diff>
--- a/website_data.xlsx
+++ b/website_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://crwindia-my.sharepoint.com/personal/fin_crwi_org_in/Documents/Jomit_clean/crwisymposium/crwisymposium-new7-4-26/crwisymposium-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="266" documentId="13_ncr:1_{43A54E2A-C15B-4049-9416-409D91501929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D62CD29-499E-4104-8244-CD7A3772FD88}"/>
+  <xr:revisionPtr revIDLastSave="282" documentId="13_ncr:1_{43A54E2A-C15B-4049-9416-409D91501929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{272F69DA-681F-49FC-ABEF-8566C276D1AA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="747" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="747" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global_Settings" sheetId="1" r:id="rId1"/>
@@ -110,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="643">
   <si>
     <t>Setting_Key</t>
   </si>
@@ -751,9 +751,6 @@
     <t>Dr. Joice Steffi Y</t>
   </si>
   <si>
-    <t>Sister</t>
-  </si>
-  <si>
     <t>Establishing sustainable and faith -rooted eldercare models that uphold diginity and independence</t>
   </si>
   <si>
@@ -871,9 +868,6 @@
     <t>MSMHC</t>
   </si>
   <si>
-    <t>St.Pauls</t>
-  </si>
-  <si>
     <t>CSsR</t>
   </si>
   <si>
@@ -1099,18 +1093,12 @@
     <t xml:space="preserve">Fr. Saju Chackalakkal </t>
   </si>
   <si>
-    <t xml:space="preserve">Fr. Jose Palely   </t>
-  </si>
-  <si>
     <t>images/Speakers/Sr. Jane.jpg</t>
   </si>
   <si>
     <t>images/Speakers/Fr. Saju.jpg</t>
   </si>
   <si>
-    <t>images/Speakers/Fr. Jose Palely.jpg</t>
-  </si>
-  <si>
     <t>Example Setting_Value</t>
   </si>
   <si>
@@ -1306,9 +1294,6 @@
     <t xml:space="preserve">Administrator Christ University </t>
   </si>
   <si>
-    <t>Vice Chancelor, ADBU, Guwahati</t>
-  </si>
-  <si>
     <t>CRI President</t>
   </si>
   <si>
@@ -1492,15 +1477,9 @@
     <t xml:space="preserve">Sr. Dr. Mary Paul </t>
   </si>
   <si>
-    <t>Fr. Dr. Sajith Cyriac, SSP</t>
-  </si>
-  <si>
     <t>SJ</t>
   </si>
   <si>
-    <t>Dr.Benny</t>
-  </si>
-  <si>
     <t>images/Presenters/modrators/Jerin.jpg</t>
   </si>
   <si>
@@ -1628,9 +1607,6 @@
   </si>
   <si>
     <t>Fr. V. Antony Bhyju, CMF, is a Claretian Missionary with wide experience in initial and ongoing formation, currently serving at the General Curia in Rome as Assistant to the General Consultors for Formation and Spirituality.</t>
-  </si>
-  <si>
-    <t>Sr. Dr. Helen Mary, SABS, is an Obstetrician and Gynecologist with an MBBS and MD from St. John’s Medical College and has served as Chief Medical Officer at Nirmala Health Centre, Bangalore, since 2002.</t>
   </si>
   <si>
     <t>Sr. Lismy CMC, of the Congregation of the Mother of Carmel, is a Catholic media missionary from Kerala, popularly known as the “Camera Nun.” She uses filmmaking and digital media for evangelization and social awareness and has produced numerous films highlighting faith, human dignity, and social issues. She is a recipient of the James Alberione Award for her contributions to Christian media.</t>
@@ -2036,6 +2012,37 @@
   </si>
   <si>
     <t>Sonia lamngaihchiin neihsiel</t>
+  </si>
+  <si>
+    <t>FDCC</t>
+  </si>
+  <si>
+    <t>SSP</t>
+  </si>
+  <si>
+    <t>Fr. Dr. Sajith Cyriac</t>
+  </si>
+  <si>
+    <t>Dr. Benny Joseph Neelankavil</t>
+  </si>
+  <si>
+    <t>CEO, Jubilee Mission Health Care Institutions</t>
+  </si>
+  <si>
+    <t>Dr. Benny Joseph Neelankavil CEO, Jubilee Mission Health Care Institutions
+Healthcare leader with 25+ years in management and academics. Oversees seven institutions including a 1,700-bed hospital. Ph.D. in Management (IIM Ahmedabad). President, AHPI Kerala Chapter; Board Member, CHAI Kerala.</t>
+  </si>
+  <si>
+    <t>Fr. Viju Painadath</t>
+  </si>
+  <si>
+    <t>Pro Vice Chancellor, Christ</t>
+  </si>
+  <si>
+    <t>images/Speakers/Dr Fr Viju P D.jpg</t>
+  </si>
+  <si>
+    <t>Sr. Dr. Helen Mary, SAB, is an Obstetrician and Gynecologist with an MBBS and MD from St. John’s Medical College and has served as Chief Medical Officer at Nirmala Health Centre, Bangalore, since 2002.</t>
   </si>
 </sst>
 </file>
@@ -2282,7 +2289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2297,9 +2304,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2395,11 +2399,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2419,6 +2419,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2844,13 +2856,13 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2903,7 +2915,7 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -2914,7 +2926,7 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -2936,22 +2948,22 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>325</v>
-      </c>
-      <c r="E9" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>437</v>
+      <c r="G9" s="6" t="s">
+        <v>432</v>
       </c>
       <c r="N9" t="s">
         <v>19</v>
@@ -2959,56 +2971,56 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="B10" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="C10" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="D10" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E10" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="H10" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I10" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="E11" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="H11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I11" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>334</v>
+      <c r="B12" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>330</v>
       </c>
       <c r="E12" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="H12" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I12" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
@@ -3016,186 +3028,186 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="C13" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="B14" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C14" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B15" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="C15" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B16" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="C16" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="B17" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C17" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="B18" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C18" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="B19" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="C19" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B20" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C20" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="B21" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="C21" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="B22" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C22" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B23" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C23" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B24" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="C24" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="B25" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C25" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="B26" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C26" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="B27" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C27" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="B28" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="C28" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="B29" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="C29" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -3318,84 +3330,84 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="C2" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="D2" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="E2" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>387</v>
+      <c r="B3" s="7" t="s">
+        <v>383</v>
       </c>
       <c r="C3" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="D3" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="E3" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>421</v>
+      <c r="B4" s="8" t="s">
+        <v>416</v>
       </c>
       <c r="C4" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="D4" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="E4" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>535</v>
+      <c r="B5" s="8" t="s">
+        <v>527</v>
       </c>
       <c r="C5" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="D5" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="E5" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>390</v>
+      <c r="B6" s="8" t="s">
+        <v>386</v>
       </c>
       <c r="C6" t="s">
+        <v>387</v>
+      </c>
+      <c r="D6" t="s">
+        <v>521</v>
+      </c>
+      <c r="E6" t="s">
         <v>391</v>
-      </c>
-      <c r="D6" t="s">
-        <v>529</v>
-      </c>
-      <c r="E6" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -3403,16 +3415,16 @@
         <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="C7" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="D7" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="E7" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -3420,16 +3432,16 @@
         <v>187</v>
       </c>
       <c r="B8" t="s">
+        <v>326</v>
+      </c>
+      <c r="C8" t="s">
+        <v>394</v>
+      </c>
+      <c r="D8" t="s">
+        <v>531</v>
+      </c>
+      <c r="E8" t="s">
         <v>328</v>
-      </c>
-      <c r="C8" t="s">
-        <v>399</v>
-      </c>
-      <c r="D8" t="s">
-        <v>539</v>
-      </c>
-      <c r="E8" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -3437,16 +3449,16 @@
         <v>191</v>
       </c>
       <c r="B9" t="s">
-        <v>329</v>
+        <v>639</v>
       </c>
       <c r="C9" t="s">
-        <v>398</v>
+        <v>640</v>
       </c>
       <c r="D9" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="E9" t="s">
-        <v>332</v>
+        <v>641</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -3454,16 +3466,16 @@
         <v>194</v>
       </c>
       <c r="B10" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="C10" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="D10" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="E10" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -3471,13 +3483,13 @@
         <v>197</v>
       </c>
       <c r="B11" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="C11" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="D11" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="E11" t="s">
         <v>163</v>
@@ -3488,16 +3500,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="C12" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="D12" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="E12" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -3505,13 +3517,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="C13" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="D13" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="E13" t="s">
         <v>166</v>
@@ -3522,16 +3534,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="C14" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="D14" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="E14" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -3576,13 +3588,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="C2" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="E2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -3590,13 +3602,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="C3" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="E3" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -3604,13 +3616,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C4" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="E4" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -3618,69 +3630,69 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="C5" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="E5" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="45" t="s">
-        <v>543</v>
+      <c r="B6" s="43" t="s">
+        <v>535</v>
       </c>
       <c r="C6" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="E6" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="45" t="s">
-        <v>544</v>
+      <c r="B7" s="43" t="s">
+        <v>536</v>
       </c>
       <c r="C7" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="E7" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="43" t="s">
-        <v>545</v>
+      <c r="B8" s="42" t="s">
+        <v>537</v>
       </c>
       <c r="C8" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="E8" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="43" t="s">
-        <v>546</v>
+      <c r="B9" s="42" t="s">
+        <v>538</v>
       </c>
       <c r="C9" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E9" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -3695,12 +3707,12 @@
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.08203125" customWidth="1"/>
+    <col min="2" max="2" width="26.08203125" style="51" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" customWidth="1"/>
     <col min="4" max="4" width="31.08203125" customWidth="1"/>
     <col min="5" max="5" width="23.25" customWidth="1"/>
     <col min="6" max="6" width="36" customWidth="1"/>
-    <col min="7" max="7" width="63.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="63.33203125" style="56" customWidth="1"/>
     <col min="8" max="8" width="9.5" customWidth="1"/>
     <col min="9" max="9" width="44.1640625" customWidth="1"/>
   </cols>
@@ -3709,7 +3721,7 @@
       <c r="A1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="51" t="s">
         <v>129</v>
       </c>
       <c r="C1" t="s">
@@ -3724,45 +3736,45 @@
       <c r="F1" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="56" t="s">
         <v>132</v>
       </c>
       <c r="H1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>615</v>
+      <c r="B2" s="51" t="s">
+        <v>607</v>
       </c>
       <c r="C2" t="s">
-        <v>616</v>
+        <v>608</v>
       </c>
       <c r="D2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E2" t="s">
         <v>88</v>
       </c>
       <c r="F2" t="s">
-        <v>463</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>518</v>
+        <v>456</v>
+      </c>
+      <c r="G2" s="56" t="s">
+        <v>510</v>
       </c>
       <c r="H2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="43" t="s">
-        <v>451</v>
+      <c r="B3" s="51" t="s">
+        <v>446</v>
       </c>
       <c r="C3" t="s">
         <v>205</v>
@@ -3774,24 +3786,24 @@
         <v>88</v>
       </c>
       <c r="F3" t="s">
-        <v>298</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>257</v>
+        <v>296</v>
+      </c>
+      <c r="G3" s="56" t="s">
+        <v>255</v>
       </c>
       <c r="H3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="43" t="s">
-        <v>547</v>
+      <c r="B4" s="51" t="s">
+        <v>539</v>
       </c>
       <c r="C4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D4" t="s">
         <v>209</v>
@@ -3800,21 +3812,21 @@
         <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>299</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>517</v>
+        <v>297</v>
+      </c>
+      <c r="G4" s="56" t="s">
+        <v>509</v>
       </c>
       <c r="H4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="43" t="s">
-        <v>620</v>
+      <c r="B5" s="51" t="s">
+        <v>612</v>
       </c>
       <c r="C5" t="s">
         <v>204</v>
@@ -3826,24 +3838,24 @@
         <v>88</v>
       </c>
       <c r="F5" t="s">
-        <v>302</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>505</v>
+        <v>300</v>
+      </c>
+      <c r="G5" s="56" t="s">
+        <v>498</v>
       </c>
       <c r="H5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="51" t="s">
         <v>202</v>
       </c>
       <c r="C6" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="D6" t="s">
         <v>211</v>
@@ -3852,852 +3864,852 @@
         <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>272</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>258</v>
+        <v>270</v>
+      </c>
+      <c r="G6" s="56" t="s">
+        <v>256</v>
       </c>
       <c r="H6" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="43" t="s">
-        <v>456</v>
+      <c r="B7" s="51" t="s">
+        <v>451</v>
       </c>
       <c r="C7" t="s">
         <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
       <c r="E7" t="s">
         <v>88</v>
       </c>
       <c r="F7" t="s">
-        <v>271</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>525</v>
+        <v>269</v>
+      </c>
+      <c r="G7" s="56" t="s">
+        <v>517</v>
       </c>
       <c r="H7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="43" t="s">
-        <v>408</v>
+      <c r="B8" s="51" t="s">
+        <v>403</v>
       </c>
       <c r="C8" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="D8" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="E8" t="s">
         <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>440</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>513</v>
+        <v>435</v>
+      </c>
+      <c r="G8" s="56" t="s">
+        <v>505</v>
       </c>
       <c r="H8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>548</v>
+      <c r="B9" s="52" t="s">
+        <v>540</v>
       </c>
       <c r="C9" t="s">
-        <v>614</v>
+        <v>606</v>
       </c>
       <c r="D9" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E9" t="s">
         <v>94</v>
       </c>
       <c r="F9" t="s">
-        <v>612</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>613</v>
+        <v>604</v>
+      </c>
+      <c r="G9" s="56" t="s">
+        <v>605</v>
       </c>
       <c r="H9" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="43" t="s">
-        <v>619</v>
+      <c r="B10" s="51" t="s">
+        <v>611</v>
       </c>
       <c r="C10" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="D10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E10" t="s">
         <v>94</v>
       </c>
       <c r="F10" t="s">
-        <v>282</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>511</v>
+        <v>280</v>
+      </c>
+      <c r="G10" s="56" t="s">
+        <v>503</v>
       </c>
       <c r="H10" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="43" t="s">
-        <v>230</v>
+      <c r="B11" s="51" t="s">
+        <v>229</v>
       </c>
       <c r="C11" t="s">
-        <v>213</v>
+        <v>633</v>
       </c>
       <c r="D11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E11" t="s">
         <v>94</v>
       </c>
       <c r="F11" t="s">
-        <v>420</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>264</v>
+        <v>415</v>
+      </c>
+      <c r="G11" s="56" t="s">
+        <v>262</v>
       </c>
       <c r="H11" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="43" t="s">
-        <v>321</v>
+      <c r="B12" s="51" t="s">
+        <v>319</v>
       </c>
       <c r="C12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D12" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E12" t="s">
         <v>94</v>
       </c>
       <c r="F12" t="s">
-        <v>284</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>510</v>
+        <v>282</v>
+      </c>
+      <c r="G12" s="56" t="s">
+        <v>502</v>
       </c>
       <c r="H12" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="43" t="s">
-        <v>231</v>
+      <c r="B13" s="51" t="s">
+        <v>230</v>
       </c>
       <c r="C13" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="D13" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E13" t="s">
         <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>286</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>265</v>
+        <v>284</v>
+      </c>
+      <c r="G13" s="56" t="s">
+        <v>263</v>
       </c>
       <c r="H13" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>549</v>
+      <c r="B14" s="52" t="s">
+        <v>541</v>
       </c>
       <c r="C14" t="s">
         <v>133</v>
       </c>
       <c r="D14" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E14" t="s">
         <v>104</v>
       </c>
       <c r="F14" t="s">
-        <v>417</v>
-      </c>
-      <c r="G14" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="G14" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H14" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="43" t="s">
-        <v>460</v>
+      <c r="B15" s="51" t="s">
+        <v>635</v>
       </c>
       <c r="C15" t="s">
+        <v>634</v>
+      </c>
+      <c r="D15" t="s">
         <v>253</v>
-      </c>
-      <c r="D15" t="s">
-        <v>255</v>
       </c>
       <c r="E15" t="s">
         <v>104</v>
       </c>
       <c r="F15" t="s">
-        <v>294</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>269</v>
+        <v>292</v>
+      </c>
+      <c r="G15" s="56" t="s">
+        <v>267</v>
       </c>
       <c r="H15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="51" t="s">
+        <v>316</v>
+      </c>
+      <c r="C16" t="s">
+        <v>251</v>
+      </c>
+      <c r="D16" t="s">
         <v>318</v>
-      </c>
-      <c r="C16" t="s">
-        <v>252</v>
-      </c>
-      <c r="D16" t="s">
-        <v>320</v>
       </c>
       <c r="E16" t="s">
         <v>104</v>
       </c>
       <c r="F16" t="s">
-        <v>293</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>256</v>
+        <v>291</v>
+      </c>
+      <c r="G16" s="56" t="s">
+        <v>254</v>
       </c>
       <c r="H16" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="93" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="43" t="s">
-        <v>250</v>
+      <c r="B17" s="51" t="s">
+        <v>249</v>
       </c>
       <c r="C17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D17" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E17" t="s">
         <v>104</v>
       </c>
       <c r="F17" t="s">
-        <v>296</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>507</v>
+        <v>294</v>
+      </c>
+      <c r="G17" s="56" t="s">
+        <v>499</v>
       </c>
       <c r="H17" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="43" t="s">
-        <v>251</v>
+      <c r="B18" s="51" t="s">
+        <v>250</v>
       </c>
       <c r="C18" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D18" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E18" t="s">
         <v>104</v>
       </c>
       <c r="F18" t="s">
-        <v>297</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>301</v>
+        <v>295</v>
+      </c>
+      <c r="G18" s="56" t="s">
+        <v>299</v>
       </c>
       <c r="H18" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
-        <v>450</v>
+      <c r="B19" s="51" t="s">
+        <v>445</v>
       </c>
       <c r="C19" t="s">
         <v>133</v>
       </c>
       <c r="D19" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E19" t="s">
         <v>91</v>
       </c>
       <c r="F19" t="s">
-        <v>464</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>514</v>
+        <v>457</v>
+      </c>
+      <c r="G19" s="56" t="s">
+        <v>506</v>
       </c>
       <c r="H19" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="43" t="s">
-        <v>457</v>
+      <c r="B20" s="51" t="s">
+        <v>452</v>
       </c>
       <c r="C20" t="s">
         <v>203</v>
       </c>
       <c r="D20" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E20" t="s">
         <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>405</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>512</v>
+        <v>400</v>
+      </c>
+      <c r="G20" s="56" t="s">
+        <v>504</v>
       </c>
       <c r="H20" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="43" t="s">
-        <v>452</v>
+      <c r="B21" s="51" t="s">
+        <v>447</v>
       </c>
       <c r="C21" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="D21" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E21" t="s">
         <v>91</v>
       </c>
       <c r="F21" t="s">
-        <v>278</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>261</v>
+        <v>276</v>
+      </c>
+      <c r="G21" s="56" t="s">
+        <v>259</v>
       </c>
       <c r="H21" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="46" t="s">
-        <v>618</v>
+      <c r="B22" s="52" t="s">
+        <v>610</v>
       </c>
       <c r="C22" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D22" t="s">
-        <v>327</v>
-      </c>
-      <c r="E22" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>524</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>617</v>
+        <v>516</v>
+      </c>
+      <c r="G22" s="56" t="s">
+        <v>609</v>
       </c>
       <c r="H22" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="43" t="s">
-        <v>221</v>
+      <c r="B23" s="51" t="s">
+        <v>220</v>
       </c>
       <c r="C23" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="D23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E23" t="s">
         <v>91</v>
       </c>
       <c r="F23" t="s">
-        <v>281</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>263</v>
+        <v>279</v>
+      </c>
+      <c r="G23" s="56" t="s">
+        <v>261</v>
       </c>
       <c r="H23" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="43" t="s">
-        <v>445</v>
+      <c r="B24" s="51" t="s">
+        <v>440</v>
       </c>
       <c r="C24" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D24" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E24" t="s">
         <v>91</v>
       </c>
       <c r="F24" t="s">
-        <v>279</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>454</v>
+        <v>277</v>
+      </c>
+      <c r="G24" s="56" t="s">
+        <v>449</v>
       </c>
       <c r="H24" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="43" t="s">
-        <v>220</v>
+      <c r="B25" s="51" t="s">
+        <v>219</v>
       </c>
       <c r="C25" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="D25" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E25" t="s">
         <v>91</v>
       </c>
       <c r="F25" t="s">
-        <v>280</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>262</v>
+        <v>278</v>
+      </c>
+      <c r="G25" s="56" t="s">
+        <v>260</v>
       </c>
       <c r="H25" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>523</v>
+      <c r="B26" s="52" t="s">
+        <v>515</v>
       </c>
       <c r="C26" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="D26" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E26" t="s">
         <v>100</v>
       </c>
       <c r="F26" t="s">
-        <v>465</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>515</v>
+        <v>458</v>
+      </c>
+      <c r="G26" s="56" t="s">
+        <v>507</v>
       </c>
       <c r="H26" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>26</v>
       </c>
-      <c r="B27" s="43" t="s">
-        <v>238</v>
+      <c r="B27" s="51" t="s">
+        <v>237</v>
       </c>
       <c r="C27" t="s">
         <v>203</v>
       </c>
       <c r="D27" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E27" t="s">
         <v>100</v>
       </c>
       <c r="F27" t="s">
-        <v>287</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>266</v>
+        <v>285</v>
+      </c>
+      <c r="G27" s="56" t="s">
+        <v>264</v>
       </c>
       <c r="H27" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="43" t="s">
-        <v>322</v>
+      <c r="B28" s="51" t="s">
+        <v>320</v>
       </c>
       <c r="C28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D28" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E28" t="s">
         <v>100</v>
       </c>
       <c r="F28" t="s">
-        <v>490</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>509</v>
+        <v>483</v>
+      </c>
+      <c r="G28" s="56" t="s">
+        <v>501</v>
       </c>
       <c r="H28" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="43" t="s">
-        <v>550</v>
+      <c r="B29" s="51" t="s">
+        <v>542</v>
       </c>
       <c r="C29" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D29" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E29" t="s">
         <v>100</v>
       </c>
       <c r="F29" t="s">
-        <v>419</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>267</v>
+        <v>414</v>
+      </c>
+      <c r="G29" s="56" t="s">
+        <v>265</v>
       </c>
       <c r="H29" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="43" t="s">
-        <v>239</v>
+      <c r="B30" s="51" t="s">
+        <v>238</v>
       </c>
       <c r="C30" t="s">
         <v>206</v>
       </c>
       <c r="D30" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E30" t="s">
         <v>100</v>
       </c>
       <c r="F30" t="s">
-        <v>292</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>268</v>
+        <v>290</v>
+      </c>
+      <c r="G30" s="56" t="s">
+        <v>266</v>
       </c>
       <c r="H30" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="43" t="s">
-        <v>551</v>
+      <c r="B31" s="51" t="s">
+        <v>543</v>
       </c>
       <c r="C31" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D31" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E31" t="s">
         <v>100</v>
       </c>
       <c r="F31" t="s">
-        <v>291</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>508</v>
+        <v>289</v>
+      </c>
+      <c r="G31" s="56" t="s">
+        <v>500</v>
       </c>
       <c r="H31" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="B32" s="44" t="s">
-        <v>455</v>
+      <c r="B32" s="53" t="s">
+        <v>450</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="D32" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E32" t="s">
         <v>100</v>
       </c>
       <c r="F32" t="s">
-        <v>288</v>
-      </c>
-      <c r="G32" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="G32" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H32" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>32</v>
       </c>
-      <c r="B33" t="s">
-        <v>462</v>
+      <c r="B33" s="51" t="s">
+        <v>636</v>
       </c>
       <c r="C33" t="s">
-        <v>133</v>
+        <v>637</v>
       </c>
       <c r="D33" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="E33" t="s">
         <v>97</v>
       </c>
       <c r="F33" t="s">
-        <v>417</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>133</v>
+        <v>412</v>
+      </c>
+      <c r="G33" s="56" t="s">
+        <v>638</v>
       </c>
       <c r="H33" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>33</v>
       </c>
-      <c r="B34" s="43" t="s">
-        <v>552</v>
+      <c r="B34" s="51" t="s">
+        <v>544</v>
       </c>
       <c r="C34" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D34" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E34" t="s">
         <v>97</v>
       </c>
       <c r="F34" t="s">
-        <v>300</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>506</v>
+        <v>298</v>
+      </c>
+      <c r="G34" s="56" t="s">
+        <v>642</v>
       </c>
       <c r="H34" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>34</v>
       </c>
-      <c r="B35" s="43" t="s">
-        <v>520</v>
+      <c r="B35" s="51" t="s">
+        <v>512</v>
       </c>
       <c r="C35" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D35" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E35" t="s">
         <v>97</v>
       </c>
       <c r="F35" t="s">
-        <v>277</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>260</v>
+        <v>275</v>
+      </c>
+      <c r="G35" s="56" t="s">
+        <v>258</v>
       </c>
       <c r="H35" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="B36" s="43" t="s">
+      <c r="B36" s="51" t="s">
         <v>212</v>
       </c>
       <c r="C36" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="D36" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E36" t="s">
         <v>97</v>
       </c>
       <c r="F36" t="s">
-        <v>275</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>260</v>
+        <v>273</v>
+      </c>
+      <c r="G36" s="56" t="s">
+        <v>258</v>
       </c>
       <c r="H36" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>36</v>
       </c>
-      <c r="B37" s="43" t="s">
-        <v>459</v>
+      <c r="B37" s="51" t="s">
+        <v>454</v>
       </c>
       <c r="C37" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D37" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E37" t="s">
         <v>97</v>
       </c>
       <c r="F37" t="s">
-        <v>273</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>259</v>
+        <v>271</v>
+      </c>
+      <c r="G37" s="56" t="s">
+        <v>257</v>
       </c>
       <c r="H37" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="62" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>37</v>
       </c>
-      <c r="B38" s="43" t="s">
-        <v>621</v>
+      <c r="B38" s="51" t="s">
+        <v>613</v>
       </c>
       <c r="C38" t="s">
         <v>206</v>
       </c>
       <c r="D38" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E38" t="s">
         <v>97</v>
       </c>
       <c r="F38" t="s">
-        <v>274</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>516</v>
+        <v>272</v>
+      </c>
+      <c r="G38" s="56" t="s">
+        <v>508</v>
       </c>
       <c r="H38" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>38</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="51" t="s">
         <v>133</v>
       </c>
       <c r="C39" t="s">
@@ -4707,151 +4719,151 @@
         <v>208</v>
       </c>
       <c r="F39" t="s">
-        <v>270</v>
-      </c>
-      <c r="G39" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="G39" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H39" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>39</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>317</v>
+      <c r="B40" s="54" t="s">
+        <v>315</v>
       </c>
       <c r="C40" t="s">
         <v>133</v>
       </c>
       <c r="D40" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E40" t="s">
         <v>97</v>
       </c>
       <c r="F40" t="s">
-        <v>276</v>
-      </c>
-      <c r="G40" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G40" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H40" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>40</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>229</v>
+      <c r="B41" s="55" t="s">
+        <v>228</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>206</v>
       </c>
       <c r="D41" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E41" t="s">
         <v>94</v>
       </c>
       <c r="F41" t="s">
-        <v>283</v>
-      </c>
-      <c r="G41" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="G41" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H41" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>317</v>
+      <c r="B42" s="54" t="s">
+        <v>315</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>133</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F42" t="s">
-        <v>285</v>
-      </c>
-      <c r="G42" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G42" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H42" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>42</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>317</v>
+      <c r="B43" s="54" t="s">
+        <v>315</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>133</v>
       </c>
       <c r="F43" t="s">
-        <v>289</v>
-      </c>
-      <c r="G43" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="G43" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H43" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>43</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>317</v>
+      <c r="B44" s="54" t="s">
+        <v>315</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>133</v>
       </c>
       <c r="F44" t="s">
-        <v>290</v>
-      </c>
-      <c r="G44" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="G44" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H44" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>44</v>
       </c>
-      <c r="B45" s="6" t="s">
-        <v>317</v>
+      <c r="B45" s="54" t="s">
+        <v>315</v>
       </c>
       <c r="C45" t="s">
         <v>133</v>
       </c>
       <c r="D45" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F45" t="s">
-        <v>295</v>
-      </c>
-      <c r="G45" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="G45" s="56" t="s">
         <v>133</v>
       </c>
       <c r="H45" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -5081,13 +5093,13 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -5095,13 +5107,13 @@
         <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C3" t="s">
         <v>150</v>
       </c>
       <c r="D3" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -5109,13 +5121,13 @@
         <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>154</v>
       </c>
       <c r="D4" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -5123,13 +5135,13 @@
         <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C5" t="s">
         <v>158</v>
       </c>
       <c r="D5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -5137,13 +5149,13 @@
         <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C6" t="s">
         <v>158</v>
       </c>
       <c r="D6" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -5151,13 +5163,13 @@
         <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C7" t="s">
         <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -5192,7 +5204,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -5203,7 +5215,7 @@
         <v>185</v>
       </c>
       <c r="C3" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D3" t="s">
         <v>85</v>
@@ -5214,13 +5226,13 @@
         <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C4" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -5231,10 +5243,10 @@
         <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -5245,10 +5257,10 @@
         <v>181</v>
       </c>
       <c r="C6" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -5256,13 +5268,13 @@
         <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="C7" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D7" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -5270,13 +5282,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
       <c r="C8" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D8" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -5284,13 +5296,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="C9" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D9" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -5298,13 +5310,13 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C10" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D10" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -5312,13 +5324,13 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="C11" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D11" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -5326,13 +5338,13 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="C12" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D12" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -5340,18 +5352,18 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="C13" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D13" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -5359,13 +5371,13 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
       <c r="C15" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D15" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -5373,13 +5385,13 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="C16" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D16" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -5387,13 +5399,13 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="C17" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D17" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -5401,13 +5413,13 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="C18" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D18" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -5415,13 +5427,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="C19" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D19" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -5429,13 +5441,13 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="C20" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D20" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -5443,13 +5455,13 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
       <c r="C21" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D21" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -5457,13 +5469,13 @@
         <v>8</v>
       </c>
       <c r="B22" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="C22" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D22" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -5471,13 +5483,13 @@
         <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="C23" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D23" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -5485,13 +5497,13 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="C24" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D24" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -5499,13 +5511,13 @@
         <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="C25" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D25" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -5513,13 +5525,13 @@
         <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>553</v>
+        <v>545</v>
       </c>
       <c r="C26" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D26" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -5527,13 +5539,13 @@
         <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="C27" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D27" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -5541,13 +5553,13 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
       <c r="C28" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D28" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -5555,13 +5567,13 @@
         <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
       <c r="C29" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D29" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
     </row>
   </sheetData>
@@ -5744,7 +5756,7 @@
         <v>196</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="E10" t="s">
         <v>128</v>
@@ -5939,7 +5951,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>51</v>
@@ -6055,303 +6067,303 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="11"/>
-      <c r="B1" s="12" t="s">
-        <v>611</v>
-      </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="A1" s="10"/>
+      <c r="B1" s="11" t="s">
+        <v>603</v>
+      </c>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
+        <v>552</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>553</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13">
+        <v>46148</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>555</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="16" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="17"/>
+      <c r="B4" s="18" t="s">
+        <v>557</v>
+      </c>
+      <c r="C4" s="19"/>
+      <c r="D4" s="20" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="13">
+        <v>46149</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>559</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>560</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="D5" s="22" t="s">
         <v>561</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="17"/>
+      <c r="B6" s="18" t="s">
         <v>562</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="14">
-        <v>46148</v>
-      </c>
-      <c r="B3" s="15" t="s">
+      <c r="C6" s="19"/>
+      <c r="D6" s="23" t="s">
         <v>563</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="18"/>
+      <c r="B7" s="18" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="18"/>
-      <c r="B4" s="19" t="s">
+      <c r="C7" s="18"/>
+      <c r="D7" s="20" t="s">
         <v>565</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="14">
-        <v>46149</v>
-      </c>
-      <c r="B5" s="22" t="s">
+      <c r="C8" s="19"/>
+      <c r="D8" s="24" t="s">
         <v>567</v>
       </c>
-      <c r="C5" s="16" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18" t="s">
         <v>568</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="C9" s="19"/>
+      <c r="D9" s="24" t="s">
         <v>569</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="18"/>
-      <c r="B6" s="19" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18" t="s">
         <v>570</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="24" t="s">
+      <c r="C10" s="19"/>
+      <c r="D10" s="24" t="s">
         <v>571</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19" t="s">
+    <row r="11" spans="1:4" ht="42.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="18"/>
+      <c r="B11" s="25" t="s">
         <v>572</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="21" t="s">
+      <c r="C11" s="19"/>
+      <c r="D11" s="24" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="19"/>
-      <c r="B8" s="19" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10" t="s">
         <v>574</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="25" t="s">
+      <c r="C12" s="10"/>
+      <c r="D12" s="26" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10" t="s">
         <v>576</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="25" t="s">
+      <c r="C13" s="10"/>
+      <c r="D13" s="26" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="26" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10" t="s">
         <v>578</v>
       </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="25" t="s">
+      <c r="C15" s="27"/>
+      <c r="D15" s="28" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="42.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="19"/>
-      <c r="B11" s="26" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10" t="s">
         <v>580</v>
       </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="25" t="s">
+      <c r="C16" s="29"/>
+      <c r="D16" s="30" t="s">
         <v>581</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="13">
+        <v>46150</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>559</v>
+      </c>
+      <c r="C17" s="31" t="s">
         <v>582</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="27" t="s">
+      <c r="D17" s="32" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10" t="s">
+        <v>562</v>
+      </c>
+      <c r="C18" s="33"/>
+      <c r="D18" s="30" t="s">
         <v>584</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="27" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11" t="s">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="10"/>
+      <c r="B19" s="34" t="s">
         <v>585</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="27" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="35" t="s">
         <v>586</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29" t="s">
+    </row>
+    <row r="20" spans="1:4" ht="42.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="10"/>
+      <c r="B20" s="36" t="s">
         <v>587</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11" t="s">
+      <c r="C20" s="37"/>
+      <c r="D20" s="38" t="s">
         <v>588</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="31" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="10"/>
+      <c r="B21" s="39" t="s">
+        <v>566</v>
+      </c>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="14">
-        <v>46150</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>567</v>
-      </c>
-      <c r="C17" s="32" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10" t="s">
         <v>590</v>
       </c>
-      <c r="D17" s="33" t="s">
+      <c r="C22" s="10"/>
+      <c r="D22" s="40" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10" t="s">
+        <v>592</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="40" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="40" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10" t="s">
         <v>570</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="31" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="11"/>
-      <c r="B19" s="35" t="s">
-        <v>593</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="36" t="s">
+      <c r="C25" s="10"/>
+      <c r="D25" s="40" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="42.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="11"/>
-      <c r="B20" s="37" t="s">
+    <row r="26" spans="1:4" ht="31" x14ac:dyDescent="0.35">
+      <c r="A26" s="10"/>
+      <c r="B26" s="41" t="s">
         <v>595</v>
       </c>
-      <c r="C20" s="38"/>
-      <c r="D20" s="39" t="s">
+      <c r="C26" s="10"/>
+      <c r="D26" s="26" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="11"/>
-      <c r="B21" s="40" t="s">
-        <v>574</v>
-      </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11" t="s">
+      <c r="C27" s="10"/>
+      <c r="D27" s="40" t="s">
         <v>598</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="41" t="s">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" s="10"/>
+      <c r="B28" s="10" t="s">
         <v>599</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11" t="s">
+      <c r="C28" s="10"/>
+      <c r="D28" s="26" t="s">
         <v>600</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="41" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11" t="s">
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" s="10"/>
+      <c r="B29" s="10" t="s">
         <v>601</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="41" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11" t="s">
-        <v>578</v>
-      </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="41" t="s">
+      <c r="C29" s="10"/>
+      <c r="D29" s="26" t="s">
         <v>602</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="A26" s="11"/>
-      <c r="B26" s="42" t="s">
-        <v>603</v>
-      </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="27" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11" t="s">
-        <v>605</v>
-      </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="41" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11" t="s">
-        <v>607</v>
-      </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="27" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11" t="s">
-        <v>609</v>
-      </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="27" t="s">
-        <v>610</v>
       </c>
     </row>
   </sheetData>
@@ -6370,118 +6382,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="48"/>
-      <c r="B1" s="48" t="s">
+      <c r="A1" s="45"/>
+      <c r="B1" s="45" t="s">
+        <v>614</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="44"/>
+      <c r="B2" s="47" t="s">
+        <v>616</v>
+      </c>
+      <c r="C2" s="48"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="44">
+        <v>1</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>617</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="31" x14ac:dyDescent="0.35">
+      <c r="A4" s="44">
+        <v>2</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>619</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="44">
+        <v>3</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>620</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="44">
+        <v>4</v>
+      </c>
+      <c r="B6" s="44" t="s">
         <v>622</v>
       </c>
-      <c r="C1" s="47" t="s">
+      <c r="C6" s="49" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="47"/>
-      <c r="B2" s="50" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="44">
+        <v>4</v>
+      </c>
+      <c r="B7" s="44" t="s">
         <v>624</v>
       </c>
-      <c r="C2" s="51"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="47">
-        <v>1</v>
-      </c>
-      <c r="B3" s="47" t="s">
+      <c r="C7" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="C3" s="47" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="44">
+        <v>5</v>
+      </c>
+      <c r="B8" s="44" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="47">
-        <v>2</v>
-      </c>
-      <c r="B4" s="49" t="s">
+      <c r="C8" s="44" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="44">
+        <v>6</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>622</v>
+      </c>
+      <c r="C9" s="45" t="s">
         <v>627</v>
       </c>
-      <c r="C4" s="47" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="47">
-        <v>3</v>
-      </c>
-      <c r="B5" s="47" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="45">
+        <v>7</v>
+      </c>
+      <c r="B10" s="44" t="s">
         <v>628</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="C10" s="44" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="47">
-        <v>4</v>
-      </c>
-      <c r="B6" s="47" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="50">
+        <v>8</v>
+      </c>
+      <c r="B11" s="50" t="s">
         <v>630</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C11" s="50" t="s">
         <v>631</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="47">
-        <v>4</v>
-      </c>
-      <c r="B7" s="47" t="s">
-        <v>632</v>
-      </c>
-      <c r="C7" s="47" t="s">
-        <v>633</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="47">
-        <v>5</v>
-      </c>
-      <c r="B8" s="47" t="s">
-        <v>634</v>
-      </c>
-      <c r="C8" s="47" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="47">
-        <v>6</v>
-      </c>
-      <c r="B9" s="47" t="s">
-        <v>630</v>
-      </c>
-      <c r="C9" s="48" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="48">
-        <v>7</v>
-      </c>
-      <c r="B10" s="47" t="s">
-        <v>636</v>
-      </c>
-      <c r="C10" s="47" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="53">
-        <v>8</v>
-      </c>
-      <c r="B11" s="53" t="s">
-        <v>638</v>
-      </c>
-      <c r="C11" s="53" t="s">
-        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>